<commit_message>
Cambios en xlsx de so
</commit_message>
<xml_diff>
--- a/Sistemas_Operativos/Ej11-TP2.xlsx
+++ b/Sistemas_Operativos/Ej11-TP2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\Facultad\2026\Primer-Cuatrimestre\Sistemas_Operativos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fernando\Desktop\Facultad\2026\Primer-Cuatrimestre\Sistemas_Operativos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4EBC5B4-C374-4DE7-A701-614DB83D74D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C75F6B03-FDCA-4FD3-8760-C1168D9A6774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FD923883-E5A2-49CD-B4C6-0568EB065424}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FD923883-E5A2-49CD-B4C6-0568EB065424}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -237,52 +237,75 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -290,30 +313,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -652,22 +651,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEB89FE4-7A5F-4F12-8080-78946FF79ABD}">
   <dimension ref="B1:BO28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.6640625" customWidth="1"/>
-    <col min="2" max="2" width="6.21875" customWidth="1"/>
-    <col min="3" max="63" width="3.109375" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="3.109375" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" customWidth="1"/>
+    <col min="3" max="63" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:67" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:67" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="BM2" s="1"/>
       <c r="BN2" s="1" t="s">
         <v>6</v>
@@ -676,22 +675,22 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="24" t="s">
+    <row r="3" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
-      <c r="L3" s="21"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="28"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
@@ -754,20 +753,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="25" t="s">
+    <row r="4" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
       <c r="M4" s="16" t="s">
         <v>2</v>
       </c>
@@ -799,28 +788,7 @@
       <c r="AM4" s="17"/>
       <c r="AN4" s="17"/>
       <c r="AO4" s="18"/>
-      <c r="AP4" s="4"/>
-      <c r="AQ4" s="4"/>
-      <c r="AR4" s="4"/>
-      <c r="AS4" s="4"/>
-      <c r="AT4" s="4"/>
-      <c r="AU4" s="4"/>
-      <c r="AV4" s="4"/>
-      <c r="AW4" s="4"/>
-      <c r="AX4" s="4"/>
-      <c r="AY4" s="4"/>
-      <c r="AZ4" s="4"/>
-      <c r="BA4" s="4"/>
-      <c r="BB4" s="4"/>
-      <c r="BC4" s="4"/>
-      <c r="BD4" s="4"/>
-      <c r="BE4" s="4"/>
-      <c r="BF4" s="4"/>
-      <c r="BG4" s="4"/>
-      <c r="BH4" s="4"/>
-      <c r="BI4" s="4"/>
-      <c r="BJ4" s="4"/>
-      <c r="BK4" s="5"/>
+      <c r="BK4" s="4"/>
       <c r="BM4" s="1" t="s">
         <v>2</v>
       </c>
@@ -832,73 +800,16 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="26" t="s">
+    <row r="5" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="4"/>
-      <c r="Y5" s="4"/>
-      <c r="Z5" s="4"/>
-      <c r="AA5" s="4"/>
-      <c r="AB5" s="4"/>
-      <c r="AC5" s="4"/>
-      <c r="AD5" s="4"/>
-      <c r="AE5" s="4"/>
-      <c r="AF5" s="4"/>
-      <c r="AG5" s="4"/>
-      <c r="AH5" s="4"/>
-      <c r="AI5" s="4"/>
-      <c r="AJ5" s="4"/>
-      <c r="AK5" s="4"/>
-      <c r="AL5" s="4"/>
-      <c r="AM5" s="4"/>
-      <c r="AN5" s="4"/>
-      <c r="AO5" s="4"/>
-      <c r="AP5" s="13" t="s">
+      <c r="AP5" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="AQ5" s="14"/>
-      <c r="AR5" s="15"/>
-      <c r="AS5" s="4"/>
-      <c r="AT5" s="4"/>
-      <c r="AU5" s="4"/>
-      <c r="AV5" s="4"/>
-      <c r="AW5" s="4"/>
-      <c r="AX5" s="4"/>
-      <c r="AY5" s="4"/>
-      <c r="AZ5" s="4"/>
-      <c r="BA5" s="4"/>
-      <c r="BB5" s="4"/>
-      <c r="BC5" s="4"/>
-      <c r="BD5" s="4"/>
-      <c r="BE5" s="4"/>
-      <c r="BF5" s="4"/>
-      <c r="BG5" s="4"/>
-      <c r="BH5" s="4"/>
-      <c r="BI5" s="4"/>
-      <c r="BJ5" s="4"/>
-      <c r="BK5" s="5"/>
+      <c r="AQ5" s="20"/>
+      <c r="AR5" s="21"/>
+      <c r="BK5" s="4"/>
       <c r="BM5" s="1" t="s">
         <v>1</v>
       </c>
@@ -910,73 +821,20 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="27" t="s">
+    <row r="6" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="4"/>
-      <c r="S6" s="4"/>
-      <c r="T6" s="4"/>
-      <c r="U6" s="4"/>
-      <c r="V6" s="4"/>
-      <c r="W6" s="4"/>
-      <c r="X6" s="4"/>
-      <c r="Y6" s="4"/>
-      <c r="Z6" s="4"/>
-      <c r="AA6" s="4"/>
-      <c r="AB6" s="4"/>
-      <c r="AC6" s="4"/>
-      <c r="AD6" s="4"/>
-      <c r="AE6" s="4"/>
-      <c r="AF6" s="4"/>
-      <c r="AG6" s="4"/>
-      <c r="AH6" s="4"/>
-      <c r="AI6" s="4"/>
-      <c r="AJ6" s="4"/>
-      <c r="AK6" s="4"/>
-      <c r="AL6" s="4"/>
-      <c r="AM6" s="4"/>
-      <c r="AN6" s="4"/>
-      <c r="AO6" s="4"/>
-      <c r="AP6" s="4"/>
-      <c r="AQ6" s="4"/>
-      <c r="AR6" s="4"/>
-      <c r="AS6" s="10" t="s">
+      <c r="AS6" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="AT6" s="11"/>
-      <c r="AU6" s="11"/>
-      <c r="AV6" s="11"/>
-      <c r="AW6" s="11"/>
-      <c r="AX6" s="11"/>
-      <c r="AY6" s="12"/>
-      <c r="AZ6" s="4"/>
-      <c r="BA6" s="4"/>
-      <c r="BB6" s="4"/>
-      <c r="BC6" s="4"/>
-      <c r="BD6" s="4"/>
-      <c r="BE6" s="4"/>
-      <c r="BF6" s="4"/>
-      <c r="BG6" s="4"/>
-      <c r="BH6" s="4"/>
-      <c r="BI6" s="4"/>
-      <c r="BJ6" s="4"/>
-      <c r="BK6" s="5"/>
+      <c r="AT6" s="23"/>
+      <c r="AU6" s="23"/>
+      <c r="AV6" s="23"/>
+      <c r="AW6" s="23"/>
+      <c r="AX6" s="23"/>
+      <c r="AY6" s="24"/>
+      <c r="BK6" s="4"/>
       <c r="BM6" s="1" t="s">
         <v>3</v>
       </c>
@@ -988,73 +846,24 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="28" t="s">
+    <row r="7" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-      <c r="P7" s="4"/>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="4"/>
-      <c r="S7" s="4"/>
-      <c r="T7" s="4"/>
-      <c r="U7" s="4"/>
-      <c r="V7" s="4"/>
-      <c r="W7" s="4"/>
-      <c r="X7" s="4"/>
-      <c r="Y7" s="4"/>
-      <c r="Z7" s="4"/>
-      <c r="AA7" s="4"/>
-      <c r="AB7" s="4"/>
-      <c r="AC7" s="4"/>
-      <c r="AD7" s="4"/>
-      <c r="AE7" s="4"/>
-      <c r="AF7" s="4"/>
-      <c r="AG7" s="4"/>
-      <c r="AH7" s="4"/>
-      <c r="AI7" s="4"/>
-      <c r="AJ7" s="4"/>
-      <c r="AK7" s="4"/>
-      <c r="AL7" s="4"/>
-      <c r="AM7" s="4"/>
-      <c r="AN7" s="4"/>
-      <c r="AO7" s="4"/>
-      <c r="AP7" s="4"/>
-      <c r="AQ7" s="4"/>
-      <c r="AR7" s="4"/>
-      <c r="AS7" s="4"/>
-      <c r="AT7" s="4"/>
-      <c r="AU7" s="4"/>
-      <c r="AV7" s="4"/>
-      <c r="AW7" s="4"/>
-      <c r="AX7" s="4"/>
-      <c r="AY7" s="4"/>
-      <c r="AZ7" s="7" t="s">
+      <c r="AZ7" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="BA7" s="8"/>
-      <c r="BB7" s="8"/>
-      <c r="BC7" s="8"/>
-      <c r="BD7" s="8"/>
-      <c r="BE7" s="8"/>
-      <c r="BF7" s="8"/>
-      <c r="BG7" s="8"/>
-      <c r="BH7" s="8"/>
-      <c r="BI7" s="8"/>
-      <c r="BJ7" s="8"/>
-      <c r="BK7" s="9"/>
+      <c r="BA7" s="25"/>
+      <c r="BB7" s="25"/>
+      <c r="BC7" s="25"/>
+      <c r="BD7" s="25"/>
+      <c r="BE7" s="25"/>
+      <c r="BF7" s="25"/>
+      <c r="BG7" s="25"/>
+      <c r="BH7" s="25"/>
+      <c r="BI7" s="25"/>
+      <c r="BJ7" s="25"/>
+      <c r="BK7" s="15"/>
       <c r="BM7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1066,198 +875,198 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="6"/>
-      <c r="C8" s="22">
+    <row r="8" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="5"/>
+      <c r="C8" s="6">
         <v>0</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="6">
         <v>1</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="7">
         <v>2</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="6">
         <v>3</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="6">
         <v>4</v>
       </c>
-      <c r="H8" s="23">
+      <c r="H8" s="7">
         <v>5</v>
       </c>
-      <c r="I8" s="22">
+      <c r="I8" s="6">
         <v>6</v>
       </c>
-      <c r="J8" s="22">
+      <c r="J8" s="6">
         <v>7</v>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="6">
         <v>8</v>
       </c>
-      <c r="L8" s="22">
+      <c r="L8" s="6">
         <v>9</v>
       </c>
-      <c r="M8" s="23">
+      <c r="M8" s="7">
         <v>10</v>
       </c>
-      <c r="N8" s="22">
+      <c r="N8" s="6">
         <v>11</v>
       </c>
-      <c r="O8" s="22">
+      <c r="O8" s="6">
         <v>12</v>
       </c>
-      <c r="P8" s="23">
+      <c r="P8" s="7">
         <v>13</v>
       </c>
-      <c r="Q8" s="22">
+      <c r="Q8" s="6">
         <v>14</v>
       </c>
-      <c r="R8" s="23">
+      <c r="R8" s="7">
         <v>15</v>
       </c>
-      <c r="S8" s="22">
+      <c r="S8" s="6">
         <v>16</v>
       </c>
-      <c r="T8" s="22">
+      <c r="T8" s="6">
         <v>17</v>
       </c>
-      <c r="U8" s="22">
+      <c r="U8" s="6">
         <v>18</v>
       </c>
-      <c r="V8" s="22">
+      <c r="V8" s="6">
         <v>19</v>
       </c>
-      <c r="W8" s="22">
+      <c r="W8" s="6">
         <v>20</v>
       </c>
-      <c r="X8" s="22">
+      <c r="X8" s="6">
         <v>21</v>
       </c>
-      <c r="Y8" s="22">
+      <c r="Y8" s="6">
         <v>22</v>
       </c>
-      <c r="Z8" s="22">
+      <c r="Z8" s="6">
         <v>23</v>
       </c>
-      <c r="AA8" s="22">
+      <c r="AA8" s="6">
         <v>24</v>
       </c>
-      <c r="AB8" s="23">
+      <c r="AB8" s="7">
         <v>25</v>
       </c>
-      <c r="AC8" s="22">
+      <c r="AC8" s="6">
         <v>26</v>
       </c>
-      <c r="AD8" s="22">
+      <c r="AD8" s="6">
         <v>27</v>
       </c>
-      <c r="AE8" s="22">
+      <c r="AE8" s="6">
         <v>28</v>
       </c>
-      <c r="AF8" s="22">
+      <c r="AF8" s="6">
         <v>29</v>
       </c>
-      <c r="AG8" s="22">
+      <c r="AG8" s="6">
         <v>30</v>
       </c>
-      <c r="AH8" s="22">
+      <c r="AH8" s="6">
         <v>31</v>
       </c>
-      <c r="AI8" s="23">
+      <c r="AI8" s="7">
         <v>32</v>
       </c>
-      <c r="AJ8" s="22">
+      <c r="AJ8" s="6">
         <v>33</v>
       </c>
-      <c r="AK8" s="22">
+      <c r="AK8" s="6">
         <v>34</v>
       </c>
-      <c r="AL8" s="22">
+      <c r="AL8" s="6">
         <v>35</v>
       </c>
-      <c r="AM8" s="22">
+      <c r="AM8" s="6">
         <v>36</v>
       </c>
-      <c r="AN8" s="22">
+      <c r="AN8" s="6">
         <v>37</v>
       </c>
-      <c r="AO8" s="23">
+      <c r="AO8" s="7">
         <v>38</v>
       </c>
-      <c r="AP8" s="22">
+      <c r="AP8" s="6">
         <v>39</v>
       </c>
-      <c r="AQ8" s="22">
+      <c r="AQ8" s="6">
         <v>40</v>
       </c>
-      <c r="AR8" s="22">
+      <c r="AR8" s="6">
         <v>41</v>
       </c>
-      <c r="AS8" s="22">
+      <c r="AS8" s="6">
         <v>42</v>
       </c>
-      <c r="AT8" s="22">
+      <c r="AT8" s="6">
         <v>43</v>
       </c>
-      <c r="AU8" s="22">
+      <c r="AU8" s="6">
         <v>44</v>
       </c>
-      <c r="AV8" s="22">
+      <c r="AV8" s="6">
         <v>45</v>
       </c>
-      <c r="AW8" s="22">
+      <c r="AW8" s="6">
         <v>46</v>
       </c>
-      <c r="AX8" s="23">
+      <c r="AX8" s="7">
         <v>47</v>
       </c>
-      <c r="AY8" s="22">
+      <c r="AY8" s="6">
         <v>48</v>
       </c>
-      <c r="AZ8" s="22">
+      <c r="AZ8" s="6">
         <v>49</v>
       </c>
-      <c r="BA8" s="22">
+      <c r="BA8" s="6">
         <v>50</v>
       </c>
-      <c r="BB8" s="22">
+      <c r="BB8" s="6">
         <v>51</v>
       </c>
-      <c r="BC8" s="23">
+      <c r="BC8" s="7">
         <v>52</v>
       </c>
-      <c r="BD8" s="22">
+      <c r="BD8" s="6">
         <v>53</v>
       </c>
-      <c r="BE8" s="22">
+      <c r="BE8" s="6">
         <v>54</v>
       </c>
-      <c r="BF8" s="22">
+      <c r="BF8" s="6">
         <v>55</v>
       </c>
-      <c r="BG8" s="22">
+      <c r="BG8" s="6">
         <v>56</v>
       </c>
-      <c r="BH8" s="22">
+      <c r="BH8" s="6">
         <v>57</v>
       </c>
-      <c r="BI8" s="22">
+      <c r="BI8" s="6">
         <v>58</v>
       </c>
-      <c r="BJ8" s="22">
+      <c r="BJ8" s="6">
         <v>59</v>
       </c>
-      <c r="BK8" s="22">
+      <c r="BK8" s="6">
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="2:67" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:67" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="BM12" s="1"/>
       <c r="BN12" s="1" t="s">
         <v>6</v>
@@ -1266,8 +1075,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="24" t="s">
+    <row r="13" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C13" s="2"/>
@@ -1281,18 +1090,18 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
-      <c r="N13" s="19" t="s">
+      <c r="N13" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="O13" s="20"/>
-      <c r="P13" s="20"/>
-      <c r="Q13" s="20"/>
-      <c r="R13" s="20"/>
-      <c r="S13" s="20"/>
-      <c r="T13" s="20"/>
-      <c r="U13" s="20"/>
-      <c r="V13" s="20"/>
-      <c r="W13" s="21"/>
+      <c r="O13" s="27"/>
+      <c r="P13" s="27"/>
+      <c r="Q13" s="27"/>
+      <c r="R13" s="27"/>
+      <c r="S13" s="27"/>
+      <c r="T13" s="27"/>
+      <c r="U13" s="27"/>
+      <c r="V13" s="27"/>
+      <c r="W13" s="28"/>
       <c r="X13" s="2" t="s">
         <v>10</v>
       </c>
@@ -1345,43 +1154,10 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="25" t="s">
+    <row r="14" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-      <c r="R14" s="4"/>
-      <c r="S14" s="4"/>
-      <c r="T14" s="4"/>
-      <c r="U14" s="4"/>
-      <c r="V14" s="4"/>
-      <c r="W14" s="4"/>
-      <c r="X14" s="4"/>
-      <c r="Y14" s="4"/>
-      <c r="Z14" s="4"/>
-      <c r="AA14" s="4"/>
-      <c r="AB14" s="4"/>
-      <c r="AC14" s="4"/>
-      <c r="AD14" s="4"/>
-      <c r="AE14" s="4"/>
-      <c r="AF14" s="4"/>
-      <c r="AG14" s="4"/>
-      <c r="AH14" s="4"/>
-      <c r="AI14" s="4"/>
       <c r="AJ14" s="16" t="s">
         <v>2</v>
       </c>
@@ -1422,75 +1198,19 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="26" t="s">
+    <row r="15" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="D15" s="14"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="4" t="s">
+      <c r="D15" s="20"/>
+      <c r="E15" s="21"/>
+      <c r="F15" t="s">
         <v>10</v>
       </c>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="4"/>
-      <c r="R15" s="4"/>
-      <c r="S15" s="4"/>
-      <c r="T15" s="4"/>
-      <c r="U15" s="4"/>
-      <c r="V15" s="4"/>
-      <c r="W15" s="4"/>
-      <c r="X15" s="4"/>
-      <c r="Y15" s="4"/>
-      <c r="Z15" s="4"/>
-      <c r="AA15" s="4"/>
-      <c r="AB15" s="4"/>
-      <c r="AC15" s="4"/>
-      <c r="AD15" s="4"/>
-      <c r="AE15" s="4"/>
-      <c r="AF15" s="4"/>
-      <c r="AG15" s="4"/>
-      <c r="AH15" s="4"/>
-      <c r="AI15" s="4"/>
-      <c r="AJ15" s="4"/>
-      <c r="AK15" s="4"/>
-      <c r="AL15" s="4"/>
-      <c r="AM15" s="4"/>
-      <c r="AN15" s="4"/>
-      <c r="AO15" s="4"/>
-      <c r="AP15" s="4"/>
-      <c r="AQ15" s="4"/>
-      <c r="AR15" s="4"/>
-      <c r="AS15" s="4"/>
-      <c r="AT15" s="4"/>
-      <c r="AU15" s="4"/>
-      <c r="AV15" s="4"/>
-      <c r="AW15" s="4"/>
-      <c r="AX15" s="4"/>
-      <c r="AY15" s="4"/>
-      <c r="AZ15" s="4"/>
-      <c r="BA15" s="4"/>
-      <c r="BB15" s="4"/>
-      <c r="BC15" s="4"/>
-      <c r="BD15" s="4"/>
-      <c r="BE15" s="4"/>
-      <c r="BF15" s="4"/>
-      <c r="BG15" s="4"/>
-      <c r="BH15" s="4"/>
-      <c r="BI15" s="4"/>
-      <c r="BJ15" s="4"/>
-      <c r="BK15" s="5"/>
+      <c r="BK15" s="4"/>
       <c r="BM15" s="1" t="s">
         <v>1</v>
       </c>
@@ -1501,154 +1221,56 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="27" t="s">
+    <row r="16" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="12"/>
-      <c r="N16" s="4" t="s">
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="24"/>
+      <c r="N16" t="s">
         <v>10</v>
       </c>
-      <c r="O16" s="4"/>
-      <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
-      <c r="R16" s="4"/>
-      <c r="S16" s="4"/>
-      <c r="T16" s="4"/>
-      <c r="U16" s="4"/>
-      <c r="V16" s="4"/>
-      <c r="W16" s="4"/>
-      <c r="X16" s="4"/>
-      <c r="Y16" s="4"/>
-      <c r="Z16" s="4"/>
-      <c r="AA16" s="4"/>
-      <c r="AB16" s="4"/>
-      <c r="AC16" s="4"/>
-      <c r="AD16" s="4"/>
-      <c r="AE16" s="4"/>
-      <c r="AF16" s="4"/>
-      <c r="AG16" s="4"/>
-      <c r="AH16" s="4"/>
-      <c r="AI16" s="4"/>
-      <c r="AJ16" s="4"/>
-      <c r="AK16" s="4"/>
-      <c r="AL16" s="4"/>
-      <c r="AM16" s="4"/>
-      <c r="AN16" s="4"/>
-      <c r="AO16" s="4"/>
-      <c r="AP16" s="4"/>
-      <c r="AQ16" s="4"/>
-      <c r="AR16" s="4"/>
-      <c r="AS16" s="4"/>
-      <c r="AT16" s="4"/>
-      <c r="AU16" s="4"/>
-      <c r="AV16" s="4"/>
-      <c r="AW16" s="4"/>
-      <c r="AX16" s="4"/>
-      <c r="AY16" s="4"/>
-      <c r="AZ16" s="4"/>
-      <c r="BA16" s="4"/>
-      <c r="BB16" s="4"/>
-      <c r="BC16" s="4"/>
-      <c r="BD16" s="4"/>
-      <c r="BE16" s="4"/>
-      <c r="BF16" s="4"/>
-      <c r="BG16" s="4"/>
-      <c r="BH16" s="4"/>
-      <c r="BI16" s="4"/>
-      <c r="BJ16" s="4"/>
-      <c r="BK16" s="5"/>
+      <c r="BK16" s="4"/>
       <c r="BM16" s="1" t="s">
         <v>3</v>
       </c>
       <c r="BN16" s="1">
         <v>4</v>
       </c>
-      <c r="BO16" s="29">
+      <c r="BO16" s="13">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="28" t="s">
+    <row r="17" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
-      <c r="N17" s="4"/>
-      <c r="O17" s="4"/>
-      <c r="P17" s="4"/>
-      <c r="Q17" s="4"/>
-      <c r="R17" s="4"/>
-      <c r="S17" s="4"/>
-      <c r="T17" s="4"/>
-      <c r="U17" s="4"/>
-      <c r="V17" s="4"/>
-      <c r="W17" s="4"/>
-      <c r="X17" s="7" t="s">
+      <c r="X17" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="Y17" s="8"/>
-      <c r="Z17" s="8"/>
-      <c r="AA17" s="8"/>
-      <c r="AB17" s="8"/>
-      <c r="AC17" s="8"/>
-      <c r="AD17" s="8"/>
-      <c r="AE17" s="8"/>
-      <c r="AF17" s="8"/>
-      <c r="AG17" s="8"/>
-      <c r="AH17" s="8"/>
-      <c r="AI17" s="9"/>
-      <c r="AJ17" s="4" t="s">
+      <c r="Y17" s="25"/>
+      <c r="Z17" s="25"/>
+      <c r="AA17" s="25"/>
+      <c r="AB17" s="25"/>
+      <c r="AC17" s="25"/>
+      <c r="AD17" s="25"/>
+      <c r="AE17" s="25"/>
+      <c r="AF17" s="25"/>
+      <c r="AG17" s="25"/>
+      <c r="AH17" s="25"/>
+      <c r="AI17" s="15"/>
+      <c r="AJ17" t="s">
         <v>10</v>
       </c>
-      <c r="AK17" s="4"/>
-      <c r="AL17" s="4"/>
-      <c r="AM17" s="4"/>
-      <c r="AN17" s="4"/>
-      <c r="AO17" s="4"/>
-      <c r="AP17" s="4"/>
-      <c r="AQ17" s="4"/>
-      <c r="AR17" s="4"/>
-      <c r="AS17" s="4"/>
-      <c r="AT17" s="4"/>
-      <c r="AU17" s="4"/>
-      <c r="AV17" s="4"/>
-      <c r="AW17" s="4"/>
-      <c r="AX17" s="4"/>
-      <c r="AY17" s="4"/>
-      <c r="AZ17" s="4"/>
-      <c r="BA17" s="4"/>
-      <c r="BB17" s="4"/>
-      <c r="BC17" s="4"/>
-      <c r="BD17" s="4"/>
-      <c r="BE17" s="4"/>
-      <c r="BF17" s="4"/>
-      <c r="BG17" s="4"/>
-      <c r="BH17" s="4"/>
-      <c r="BI17" s="4"/>
-      <c r="BJ17" s="4"/>
-      <c r="BK17" s="5"/>
+      <c r="BK17" s="4"/>
       <c r="BM17" s="1" t="s">
         <v>4</v>
       </c>
@@ -1659,206 +1281,206 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="6"/>
-      <c r="C18" s="22">
+    <row r="18" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="5"/>
+      <c r="C18" s="6">
         <v>0</v>
       </c>
-      <c r="D18" s="22">
+      <c r="D18" s="6">
         <v>1</v>
       </c>
-      <c r="E18" s="23">
+      <c r="E18" s="7">
         <v>2</v>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="6">
         <v>3</v>
       </c>
-      <c r="G18" s="22">
+      <c r="G18" s="6">
         <v>4</v>
       </c>
-      <c r="H18" s="23">
+      <c r="H18" s="7">
         <v>5</v>
       </c>
-      <c r="I18" s="22">
+      <c r="I18" s="6">
         <v>6</v>
       </c>
-      <c r="J18" s="22">
+      <c r="J18" s="6">
         <v>7</v>
       </c>
-      <c r="K18" s="22">
+      <c r="K18" s="6">
         <v>8</v>
       </c>
-      <c r="L18" s="22">
+      <c r="L18" s="6">
         <v>9</v>
       </c>
-      <c r="M18" s="23">
+      <c r="M18" s="7">
         <v>10</v>
       </c>
-      <c r="N18" s="22">
+      <c r="N18" s="6">
         <v>11</v>
       </c>
-      <c r="O18" s="22">
+      <c r="O18" s="6">
         <v>12</v>
       </c>
-      <c r="P18" s="23">
+      <c r="P18" s="7">
         <v>13</v>
       </c>
-      <c r="Q18" s="22">
+      <c r="Q18" s="6">
         <v>14</v>
       </c>
-      <c r="R18" s="23">
+      <c r="R18" s="7">
         <v>15</v>
       </c>
-      <c r="S18" s="22">
+      <c r="S18" s="6">
         <v>16</v>
       </c>
-      <c r="T18" s="22">
+      <c r="T18" s="6">
         <v>17</v>
       </c>
-      <c r="U18" s="22">
+      <c r="U18" s="6">
         <v>18</v>
       </c>
-      <c r="V18" s="22">
+      <c r="V18" s="6">
         <v>19</v>
       </c>
-      <c r="W18" s="22">
+      <c r="W18" s="6">
         <v>20</v>
       </c>
-      <c r="X18" s="22">
+      <c r="X18" s="6">
         <v>21</v>
       </c>
-      <c r="Y18" s="22">
+      <c r="Y18" s="6">
         <v>22</v>
       </c>
-      <c r="Z18" s="22">
+      <c r="Z18" s="6">
         <v>23</v>
       </c>
-      <c r="AA18" s="22">
+      <c r="AA18" s="6">
         <v>24</v>
       </c>
-      <c r="AB18" s="23">
+      <c r="AB18" s="7">
         <v>25</v>
       </c>
-      <c r="AC18" s="22">
+      <c r="AC18" s="6">
         <v>26</v>
       </c>
-      <c r="AD18" s="22">
+      <c r="AD18" s="6">
         <v>27</v>
       </c>
-      <c r="AE18" s="22">
+      <c r="AE18" s="6">
         <v>28</v>
       </c>
-      <c r="AF18" s="22">
+      <c r="AF18" s="6">
         <v>29</v>
       </c>
-      <c r="AG18" s="22">
+      <c r="AG18" s="6">
         <v>30</v>
       </c>
-      <c r="AH18" s="22">
+      <c r="AH18" s="6">
         <v>31</v>
       </c>
-      <c r="AI18" s="23">
+      <c r="AI18" s="7">
         <v>32</v>
       </c>
-      <c r="AJ18" s="22">
+      <c r="AJ18" s="6">
         <v>33</v>
       </c>
-      <c r="AK18" s="22">
+      <c r="AK18" s="6">
         <v>34</v>
       </c>
-      <c r="AL18" s="22">
+      <c r="AL18" s="6">
         <v>35</v>
       </c>
-      <c r="AM18" s="22">
+      <c r="AM18" s="6">
         <v>36</v>
       </c>
-      <c r="AN18" s="22">
+      <c r="AN18" s="6">
         <v>37</v>
       </c>
-      <c r="AO18" s="23">
+      <c r="AO18" s="7">
         <v>38</v>
       </c>
-      <c r="AP18" s="22">
+      <c r="AP18" s="6">
         <v>39</v>
       </c>
-      <c r="AQ18" s="22">
+      <c r="AQ18" s="6">
         <v>40</v>
       </c>
-      <c r="AR18" s="22">
+      <c r="AR18" s="6">
         <v>41</v>
       </c>
-      <c r="AS18" s="22">
+      <c r="AS18" s="6">
         <v>42</v>
       </c>
-      <c r="AT18" s="22">
+      <c r="AT18" s="6">
         <v>43</v>
       </c>
-      <c r="AU18" s="22">
+      <c r="AU18" s="6">
         <v>44</v>
       </c>
-      <c r="AV18" s="22">
+      <c r="AV18" s="6">
         <v>45</v>
       </c>
-      <c r="AW18" s="22">
+      <c r="AW18" s="6">
         <v>46</v>
       </c>
-      <c r="AX18" s="23">
+      <c r="AX18" s="7">
         <v>47</v>
       </c>
-      <c r="AY18" s="22">
+      <c r="AY18" s="6">
         <v>48</v>
       </c>
-      <c r="AZ18" s="22">
+      <c r="AZ18" s="6">
         <v>49</v>
       </c>
-      <c r="BA18" s="22">
+      <c r="BA18" s="6">
         <v>50</v>
       </c>
-      <c r="BB18" s="22">
+      <c r="BB18" s="6">
         <v>51</v>
       </c>
-      <c r="BC18" s="23">
+      <c r="BC18" s="7">
         <v>52</v>
       </c>
-      <c r="BD18" s="22">
+      <c r="BD18" s="6">
         <v>53</v>
       </c>
-      <c r="BE18" s="22">
+      <c r="BE18" s="6">
         <v>54</v>
       </c>
-      <c r="BF18" s="22">
+      <c r="BF18" s="6">
         <v>55</v>
       </c>
-      <c r="BG18" s="22">
+      <c r="BG18" s="6">
         <v>56</v>
       </c>
-      <c r="BH18" s="22">
+      <c r="BH18" s="6">
         <v>57</v>
       </c>
-      <c r="BI18" s="22">
+      <c r="BI18" s="6">
         <v>58</v>
       </c>
-      <c r="BJ18" s="22">
+      <c r="BJ18" s="6">
         <v>59</v>
       </c>
-      <c r="BK18" s="22">
+      <c r="BK18" s="6">
         <v>60</v>
       </c>
       <c r="BM18" s="1"/>
       <c r="BN18" s="1"/>
       <c r="BO18" s="1"/>
     </row>
-    <row r="19" spans="2:67" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:67" x14ac:dyDescent="0.25">
       <c r="BM19" s="1"/>
       <c r="BN19" s="1"/>
       <c r="BO19" s="1"/>
     </row>
-    <row r="20" spans="2:67" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:67" x14ac:dyDescent="0.25">
       <c r="BM20" s="1"/>
       <c r="BN20" s="1"/>
       <c r="BO20" s="1"/>
     </row>
-    <row r="21" spans="2:67" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:67" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>9</v>
       </c>
@@ -1866,7 +1488,7 @@
       <c r="BN21" s="1"/>
       <c r="BO21" s="1"/>
     </row>
-    <row r="22" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="BM22" s="1"/>
       <c r="BN22" s="1" t="s">
         <v>6</v>
@@ -1875,22 +1497,22 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="24" t="s">
+    <row r="23" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20"/>
-      <c r="L23" s="21"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="28"/>
       <c r="M23" s="2" t="s">
         <v>10</v>
       </c>
@@ -1954,20 +1576,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="25" t="s">
+    <row r="24" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
-      <c r="L24" s="4"/>
       <c r="M24" s="16" t="s">
         <v>2</v>
       </c>
@@ -1980,29 +1592,9 @@
       <c r="T24" s="17"/>
       <c r="U24" s="17"/>
       <c r="V24" s="18"/>
-      <c r="W24" s="4" t="s">
+      <c r="W24" t="s">
         <v>11</v>
       </c>
-      <c r="X24" s="4"/>
-      <c r="Y24" s="4"/>
-      <c r="Z24" s="4"/>
-      <c r="AA24" s="4"/>
-      <c r="AB24" s="4"/>
-      <c r="AC24" s="4"/>
-      <c r="AD24" s="4"/>
-      <c r="AE24" s="4"/>
-      <c r="AF24" s="4"/>
-      <c r="AG24" s="4"/>
-      <c r="AH24" s="4"/>
-      <c r="AI24" s="4"/>
-      <c r="AJ24" s="4"/>
-      <c r="AK24" s="4"/>
-      <c r="AL24" s="4"/>
-      <c r="AM24" s="4"/>
-      <c r="AN24" s="4"/>
-      <c r="AO24" s="4"/>
-      <c r="AP24" s="4"/>
-      <c r="AQ24" s="4"/>
       <c r="AR24" s="16" t="s">
         <v>2</v>
       </c>
@@ -2015,10 +1607,9 @@
       <c r="AY24" s="17"/>
       <c r="AZ24" s="17"/>
       <c r="BA24" s="18"/>
-      <c r="BB24" s="4" t="s">
+      <c r="BB24" t="s">
         <v>11</v>
       </c>
-      <c r="BC24" s="4"/>
       <c r="BD24" s="16" t="s">
         <v>2</v>
       </c>
@@ -2039,75 +1630,19 @@
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="26" t="s">
+    <row r="25" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
-      <c r="L25" s="4"/>
-      <c r="M25" s="4"/>
-      <c r="N25" s="4"/>
-      <c r="O25" s="4"/>
-      <c r="P25" s="4"/>
-      <c r="Q25" s="4"/>
-      <c r="R25" s="4"/>
-      <c r="S25" s="4"/>
-      <c r="T25" s="4"/>
-      <c r="U25" s="4"/>
-      <c r="V25" s="4"/>
-      <c r="W25" s="13" t="s">
+      <c r="W25" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="X25" s="14"/>
-      <c r="Y25" s="15"/>
-      <c r="Z25" s="4" t="s">
+      <c r="X25" s="20"/>
+      <c r="Y25" s="21"/>
+      <c r="Z25" t="s">
         <v>10</v>
       </c>
-      <c r="AA25" s="4"/>
-      <c r="AB25" s="4"/>
-      <c r="AC25" s="4"/>
-      <c r="AD25" s="4"/>
-      <c r="AE25" s="4"/>
-      <c r="AF25" s="4"/>
-      <c r="AG25" s="4"/>
-      <c r="AH25" s="4"/>
-      <c r="AI25" s="4"/>
-      <c r="AJ25" s="4"/>
-      <c r="AK25" s="4"/>
-      <c r="AL25" s="4"/>
-      <c r="AM25" s="4"/>
-      <c r="AN25" s="4"/>
-      <c r="AO25" s="4"/>
-      <c r="AP25" s="4"/>
-      <c r="AQ25" s="4"/>
-      <c r="AR25" s="4"/>
-      <c r="AS25" s="4"/>
-      <c r="AT25" s="4"/>
-      <c r="AU25" s="4"/>
-      <c r="AV25" s="4"/>
-      <c r="AW25" s="4"/>
-      <c r="AX25" s="4"/>
-      <c r="AY25" s="4"/>
-      <c r="AZ25" s="4"/>
-      <c r="BA25" s="4"/>
-      <c r="BB25" s="4"/>
-      <c r="BC25" s="4"/>
-      <c r="BD25" s="4"/>
-      <c r="BE25" s="4"/>
-      <c r="BF25" s="4"/>
-      <c r="BG25" s="4"/>
-      <c r="BH25" s="4"/>
-      <c r="BI25" s="4"/>
-      <c r="BJ25" s="4"/>
-      <c r="BK25" s="5"/>
+      <c r="BK25" s="4"/>
       <c r="BM25" s="1" t="s">
         <v>1</v>
       </c>
@@ -2118,75 +1653,23 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="27" t="s">
+    <row r="26" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
-      <c r="M26" s="4"/>
-      <c r="N26" s="4"/>
-      <c r="O26" s="4"/>
-      <c r="P26" s="4"/>
-      <c r="Q26" s="4"/>
-      <c r="R26" s="4"/>
-      <c r="S26" s="4"/>
-      <c r="T26" s="4"/>
-      <c r="U26" s="4"/>
-      <c r="V26" s="4"/>
-      <c r="W26" s="4"/>
-      <c r="X26" s="4"/>
-      <c r="Y26" s="4"/>
-      <c r="Z26" s="10" t="s">
+      <c r="Z26" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="AA26" s="11"/>
-      <c r="AB26" s="11"/>
-      <c r="AC26" s="11"/>
-      <c r="AD26" s="11"/>
-      <c r="AE26" s="11"/>
-      <c r="AF26" s="12"/>
-      <c r="AG26" s="4" t="s">
+      <c r="AA26" s="23"/>
+      <c r="AB26" s="23"/>
+      <c r="AC26" s="23"/>
+      <c r="AD26" s="23"/>
+      <c r="AE26" s="23"/>
+      <c r="AF26" s="24"/>
+      <c r="AG26" t="s">
         <v>10</v>
       </c>
-      <c r="AH26" s="4"/>
-      <c r="AI26" s="4"/>
-      <c r="AJ26" s="4"/>
-      <c r="AK26" s="4"/>
-      <c r="AL26" s="4"/>
-      <c r="AM26" s="4"/>
-      <c r="AN26" s="4"/>
-      <c r="AO26" s="4"/>
-      <c r="AP26" s="4"/>
-      <c r="AQ26" s="4"/>
-      <c r="AR26" s="4"/>
-      <c r="AS26" s="4"/>
-      <c r="AT26" s="4"/>
-      <c r="AU26" s="4"/>
-      <c r="AV26" s="4"/>
-      <c r="AW26" s="4"/>
-      <c r="AX26" s="4"/>
-      <c r="AY26" s="4"/>
-      <c r="AZ26" s="4"/>
-      <c r="BA26" s="4"/>
-      <c r="BB26" s="4"/>
-      <c r="BC26" s="4"/>
-      <c r="BD26" s="4"/>
-      <c r="BE26" s="4"/>
-      <c r="BF26" s="4"/>
-      <c r="BG26" s="4"/>
-      <c r="BH26" s="4"/>
-      <c r="BI26" s="4"/>
-      <c r="BJ26" s="4"/>
-      <c r="BK26" s="5"/>
+      <c r="BK26" s="4"/>
       <c r="BM26" s="1" t="s">
         <v>3</v>
       </c>
@@ -2197,79 +1680,34 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="28" t="s">
+    <row r="27" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
-      <c r="M27" s="4"/>
-      <c r="N27" s="4"/>
-      <c r="O27" s="4"/>
-      <c r="P27" s="4"/>
-      <c r="Q27" s="4"/>
-      <c r="R27" s="4"/>
-      <c r="S27" s="4"/>
-      <c r="T27" s="4"/>
-      <c r="U27" s="4"/>
-      <c r="V27" s="4"/>
-      <c r="W27" s="4"/>
-      <c r="X27" s="4"/>
-      <c r="Y27" s="4"/>
-      <c r="Z27" s="4"/>
-      <c r="AA27" s="4"/>
-      <c r="AB27" s="4"/>
-      <c r="AC27" s="4"/>
-      <c r="AD27" s="4"/>
-      <c r="AE27" s="4"/>
-      <c r="AF27" s="4"/>
-      <c r="AG27" s="7" t="s">
+      <c r="AG27" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="AH27" s="8"/>
-      <c r="AI27" s="8"/>
-      <c r="AJ27" s="8"/>
-      <c r="AK27" s="8"/>
-      <c r="AL27" s="8"/>
-      <c r="AM27" s="8"/>
-      <c r="AN27" s="8"/>
-      <c r="AO27" s="8"/>
-      <c r="AP27" s="8"/>
-      <c r="AQ27" s="9"/>
-      <c r="AR27" s="4" t="s">
+      <c r="AH27" s="25"/>
+      <c r="AI27" s="25"/>
+      <c r="AJ27" s="25"/>
+      <c r="AK27" s="25"/>
+      <c r="AL27" s="25"/>
+      <c r="AM27" s="25"/>
+      <c r="AN27" s="25"/>
+      <c r="AO27" s="25"/>
+      <c r="AP27" s="25"/>
+      <c r="AQ27" s="15"/>
+      <c r="AR27" t="s">
         <v>11</v>
       </c>
-      <c r="AS27" s="4"/>
-      <c r="AT27" s="4"/>
-      <c r="AU27" s="4"/>
-      <c r="AV27" s="4"/>
-      <c r="AW27" s="4"/>
-      <c r="AX27" s="4"/>
-      <c r="AY27" s="4"/>
-      <c r="AZ27" s="4"/>
-      <c r="BA27" s="4"/>
-      <c r="BB27" s="7" t="s">
+      <c r="BB27" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="BC27" s="9"/>
-      <c r="BD27" s="4" t="s">
+      <c r="BC27" s="15"/>
+      <c r="BD27" t="s">
         <v>10</v>
       </c>
-      <c r="BE27" s="4"/>
-      <c r="BF27" s="4"/>
-      <c r="BG27" s="4"/>
-      <c r="BH27" s="4"/>
-      <c r="BI27" s="4"/>
-      <c r="BJ27" s="4"/>
-      <c r="BK27" s="5"/>
+      <c r="BK27" s="4"/>
       <c r="BM27" s="1" t="s">
         <v>4</v>
       </c>
@@ -2280,194 +1718,205 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="2:67" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="6"/>
-      <c r="C28" s="22">
+    <row r="28" spans="2:67" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="5"/>
+      <c r="C28" s="6">
         <v>0</v>
       </c>
-      <c r="D28" s="22">
+      <c r="D28" s="6">
         <v>1</v>
       </c>
-      <c r="E28" s="23">
+      <c r="E28" s="7">
         <v>2</v>
       </c>
-      <c r="F28" s="22">
+      <c r="F28" s="6">
         <v>3</v>
       </c>
-      <c r="G28" s="22">
+      <c r="G28" s="6">
         <v>4</v>
       </c>
-      <c r="H28" s="23">
+      <c r="H28" s="7">
         <v>5</v>
       </c>
-      <c r="I28" s="22">
+      <c r="I28" s="6">
         <v>6</v>
       </c>
-      <c r="J28" s="22">
+      <c r="J28" s="6">
         <v>7</v>
       </c>
-      <c r="K28" s="22">
+      <c r="K28" s="6">
         <v>8</v>
       </c>
-      <c r="L28" s="22">
+      <c r="L28" s="6">
         <v>9</v>
       </c>
-      <c r="M28" s="23">
+      <c r="M28" s="7">
         <v>10</v>
       </c>
-      <c r="N28" s="22">
+      <c r="N28" s="6">
         <v>11</v>
       </c>
-      <c r="O28" s="22">
+      <c r="O28" s="6">
         <v>12</v>
       </c>
-      <c r="P28" s="23">
+      <c r="P28" s="7">
         <v>13</v>
       </c>
-      <c r="Q28" s="22">
+      <c r="Q28" s="6">
         <v>14</v>
       </c>
-      <c r="R28" s="23">
+      <c r="R28" s="7">
         <v>15</v>
       </c>
-      <c r="S28" s="22">
+      <c r="S28" s="6">
         <v>16</v>
       </c>
-      <c r="T28" s="22">
+      <c r="T28" s="6">
         <v>17</v>
       </c>
-      <c r="U28" s="22">
+      <c r="U28" s="6">
         <v>18</v>
       </c>
-      <c r="V28" s="22">
+      <c r="V28" s="6">
         <v>19</v>
       </c>
-      <c r="W28" s="22">
+      <c r="W28" s="6">
         <v>20</v>
       </c>
-      <c r="X28" s="22">
+      <c r="X28" s="6">
         <v>21</v>
       </c>
-      <c r="Y28" s="22">
+      <c r="Y28" s="6">
         <v>22</v>
       </c>
-      <c r="Z28" s="22">
+      <c r="Z28" s="6">
         <v>23</v>
       </c>
-      <c r="AA28" s="22">
+      <c r="AA28" s="6">
         <v>24</v>
       </c>
-      <c r="AB28" s="23">
+      <c r="AB28" s="7">
         <v>25</v>
       </c>
-      <c r="AC28" s="22">
+      <c r="AC28" s="6">
         <v>26</v>
       </c>
-      <c r="AD28" s="22">
+      <c r="AD28" s="6">
         <v>27</v>
       </c>
-      <c r="AE28" s="22">
+      <c r="AE28" s="6">
         <v>28</v>
       </c>
-      <c r="AF28" s="22">
+      <c r="AF28" s="6">
         <v>29</v>
       </c>
-      <c r="AG28" s="22">
+      <c r="AG28" s="6">
         <v>30</v>
       </c>
-      <c r="AH28" s="22">
+      <c r="AH28" s="6">
         <v>31</v>
       </c>
-      <c r="AI28" s="23">
+      <c r="AI28" s="7">
         <v>32</v>
       </c>
-      <c r="AJ28" s="22">
+      <c r="AJ28" s="6">
         <v>33</v>
       </c>
-      <c r="AK28" s="22">
+      <c r="AK28" s="6">
         <v>34</v>
       </c>
-      <c r="AL28" s="22">
+      <c r="AL28" s="6">
         <v>35</v>
       </c>
-      <c r="AM28" s="22">
+      <c r="AM28" s="6">
         <v>36</v>
       </c>
-      <c r="AN28" s="22">
+      <c r="AN28" s="6">
         <v>37</v>
       </c>
-      <c r="AO28" s="23">
+      <c r="AO28" s="7">
         <v>38</v>
       </c>
-      <c r="AP28" s="22">
+      <c r="AP28" s="6">
         <v>39</v>
       </c>
-      <c r="AQ28" s="22">
+      <c r="AQ28" s="6">
         <v>40</v>
       </c>
-      <c r="AR28" s="22">
+      <c r="AR28" s="6">
         <v>41</v>
       </c>
-      <c r="AS28" s="22">
+      <c r="AS28" s="6">
         <v>42</v>
       </c>
-      <c r="AT28" s="22">
+      <c r="AT28" s="6">
         <v>43</v>
       </c>
-      <c r="AU28" s="22">
+      <c r="AU28" s="6">
         <v>44</v>
       </c>
-      <c r="AV28" s="22">
+      <c r="AV28" s="6">
         <v>45</v>
       </c>
-      <c r="AW28" s="22">
+      <c r="AW28" s="6">
         <v>46</v>
       </c>
-      <c r="AX28" s="23">
+      <c r="AX28" s="7">
         <v>47</v>
       </c>
-      <c r="AY28" s="22">
+      <c r="AY28" s="6">
         <v>48</v>
       </c>
-      <c r="AZ28" s="22">
+      <c r="AZ28" s="6">
         <v>49</v>
       </c>
-      <c r="BA28" s="22">
+      <c r="BA28" s="6">
         <v>50</v>
       </c>
-      <c r="BB28" s="22">
+      <c r="BB28" s="6">
         <v>51</v>
       </c>
-      <c r="BC28" s="23">
+      <c r="BC28" s="7">
         <v>52</v>
       </c>
-      <c r="BD28" s="22">
+      <c r="BD28" s="6">
         <v>53</v>
       </c>
-      <c r="BE28" s="22">
+      <c r="BE28" s="6">
         <v>54</v>
       </c>
-      <c r="BF28" s="22">
+      <c r="BF28" s="6">
         <v>55</v>
       </c>
-      <c r="BG28" s="22">
+      <c r="BG28" s="6">
         <v>56</v>
       </c>
-      <c r="BH28" s="22">
+      <c r="BH28" s="6">
         <v>57</v>
       </c>
-      <c r="BI28" s="22">
+      <c r="BI28" s="6">
         <v>58</v>
       </c>
-      <c r="BJ28" s="22">
+      <c r="BJ28" s="6">
         <v>59</v>
       </c>
-      <c r="BK28" s="22">
+      <c r="BK28" s="6">
         <v>60</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C3:L3"/>
+    <mergeCell ref="M4:AO4"/>
+    <mergeCell ref="AP5:AR5"/>
+    <mergeCell ref="AS6:AY6"/>
+    <mergeCell ref="AZ7:BK7"/>
+    <mergeCell ref="F16:M16"/>
+    <mergeCell ref="N13:W13"/>
+    <mergeCell ref="X17:AI17"/>
+    <mergeCell ref="AJ14:BK14"/>
+    <mergeCell ref="C23:L23"/>
+    <mergeCell ref="C15:E15"/>
     <mergeCell ref="BB27:BC27"/>
     <mergeCell ref="BD24:BK24"/>
     <mergeCell ref="M24:V24"/>
@@ -2475,17 +1924,6 @@
     <mergeCell ref="Z26:AF26"/>
     <mergeCell ref="AG27:AQ27"/>
     <mergeCell ref="AR24:BA24"/>
-    <mergeCell ref="F16:M16"/>
-    <mergeCell ref="N13:W13"/>
-    <mergeCell ref="X17:AI17"/>
-    <mergeCell ref="AJ14:BK14"/>
-    <mergeCell ref="C23:L23"/>
-    <mergeCell ref="C3:L3"/>
-    <mergeCell ref="M4:AO4"/>
-    <mergeCell ref="AP5:AR5"/>
-    <mergeCell ref="AS6:AY6"/>
-    <mergeCell ref="AZ7:BK7"/>
-    <mergeCell ref="C15:E15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>